<commit_message>
Update GUA IPPU model files
</commit_message>
<xml_diff>
--- a/GUA/IPPU/A1_Inputs/A-I_Classifier_Modes_Demand.xlsx
+++ b/GUA/IPPU/A1_Inputs/A-I_Classifier_Modes_Demand.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanc\Desktop\GUA_Modelos_Sectoriales\M0_IPPU_V2\A1_Inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IgnacioAlfaroCorrale\Desktop\Models_running\0_guatemala_2025\IPPU_GUA_v1_2025\A1_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA0E384-4504-4F54-9ADA-1931164DC239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C5D774-788A-4FEE-8B65-1B58EB026C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,12 @@
     <sheet name="Fuel_per_Sectors" sheetId="3" r:id="rId3"/>
     <sheet name="Fuel_to_Code" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Fuel_per_Sectors!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Fuel_to_Code!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sectors!$A$1:$C$1</definedName>
+  </definedNames>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,6 +34,9 @@
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,87 +44,201 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="65">
+  <si>
+    <t>This file will lay out the blocks of demand that are General (measured in Joules).</t>
+  </si>
   <si>
     <t>It will also indicate what parts of the RES have a specil buildup, like transport, or eventually industry.</t>
   </si>
   <si>
+    <t>Sector</t>
+  </si>
+  <si>
     <t>Plain English</t>
   </si>
   <si>
-    <t>Plain Spanish</t>
-  </si>
-  <si>
-    <t>Sector</t>
-  </si>
-  <si>
     <t>Address_Method</t>
   </si>
   <si>
     <t>Simple</t>
   </si>
   <si>
+    <t>IPPU</t>
+  </si>
+  <si>
+    <t>Industrial Processes</t>
+  </si>
+  <si>
     <t>Fuel/Sector</t>
   </si>
   <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Raw_materials_for_clinker</t>
+  </si>
+  <si>
+    <t>Raw_materials_for_cement</t>
+  </si>
+  <si>
+    <t>Clinker_production</t>
+  </si>
+  <si>
+    <t>Cement_production</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
     <t>Code</t>
   </si>
   <si>
-    <t>Fuel</t>
-  </si>
-  <si>
-    <t>This file will lay out the blocks of demand that are General (measured in Tons).</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>Raw_materials_for_clinker</t>
+    <t>RAW_MAT_CLK</t>
   </si>
   <si>
     <t>Raw materials for clinker</t>
   </si>
   <si>
-    <t>Raw_materials_for_cement</t>
+    <t>RAW_MAT_CEM</t>
   </si>
   <si>
     <t>Raw materials for cement</t>
   </si>
   <si>
-    <t>Materia prima para cemento</t>
-  </si>
-  <si>
-    <t>Materia prima para clinker</t>
-  </si>
-  <si>
-    <t>RAW_MAT_CLK</t>
-  </si>
-  <si>
-    <t>RAW_MAT_CEM</t>
-  </si>
-  <si>
-    <t>Clinker_production</t>
+    <t>CLK_PROD</t>
   </si>
   <si>
     <t>Clinker production</t>
   </si>
   <si>
+    <t>CEM_PROD</t>
+  </si>
+  <si>
     <t>Cement production</t>
   </si>
   <si>
-    <t>Cement_production</t>
-  </si>
-  <si>
-    <t>CLK_PROD</t>
-  </si>
-  <si>
-    <t>CEM_PROD</t>
-  </si>
-  <si>
-    <t>Producción de clinker</t>
-  </si>
-  <si>
-    <t>Producción de cemento</t>
+    <t>IND</t>
+  </si>
+  <si>
+    <t>Industrial</t>
+  </si>
+  <si>
+    <t>Use_Paraffin_Wax</t>
+  </si>
+  <si>
+    <t>PARAFFIN</t>
+  </si>
+  <si>
+    <t>Use of Paraffin Wax</t>
+  </si>
+  <si>
+    <t>Use_Lubricants_oils</t>
+  </si>
+  <si>
+    <t>LUBRI_OILS</t>
+  </si>
+  <si>
+    <t>Use of Lubricants Oils</t>
+  </si>
+  <si>
+    <t>Refrigeration_and_air_conditioning_HFC32</t>
+  </si>
+  <si>
+    <t>Refrigeration_and_air_conditioning_HFC125</t>
+  </si>
+  <si>
+    <t>Refrigeration_and_air_conditioning_HFC134a</t>
+  </si>
+  <si>
+    <t>Refrigeration_and_air_conditioning_HFC143a</t>
+  </si>
+  <si>
+    <t>REFR_AC_HFC32</t>
+  </si>
+  <si>
+    <t>REFR_AC_HFC125</t>
+  </si>
+  <si>
+    <t>REFR_AC_HFC134a</t>
+  </si>
+  <si>
+    <t>REFR_AC_HFC143a</t>
+  </si>
+  <si>
+    <t>Refrigeration and air conditioning HFC32</t>
+  </si>
+  <si>
+    <t>Refrigeration and air conditioning HFC125</t>
+  </si>
+  <si>
+    <t>Refrigeration and air conditioning HFC134a</t>
+  </si>
+  <si>
+    <t>Refrigeration and air conditioning HFC143a</t>
+  </si>
+  <si>
+    <t>Ferroalloy_production</t>
+  </si>
+  <si>
+    <t>PROD_FERRO</t>
+  </si>
+  <si>
+    <t>Ferroalloy production</t>
+  </si>
+  <si>
+    <t>Glass_production</t>
+  </si>
+  <si>
+    <t>GLASS_PROD</t>
+  </si>
+  <si>
+    <t>Glass production</t>
+  </si>
+  <si>
+    <t>Iron_Steel_production</t>
+  </si>
+  <si>
+    <t>IRON_STEEL</t>
+  </si>
+  <si>
+    <t>Iron and Steel production</t>
+  </si>
+  <si>
+    <t>Lime_production_calcitic</t>
+  </si>
+  <si>
+    <t>Lime_production_dolomitic</t>
+  </si>
+  <si>
+    <t>Carbonate_ceramics</t>
+  </si>
+  <si>
+    <t>Carbonate_soda_ash</t>
+  </si>
+  <si>
+    <t>LIME_CAL_PROD</t>
+  </si>
+  <si>
+    <t>LIME_DOL_PROD</t>
+  </si>
+  <si>
+    <t>Lime production calcitic</t>
+  </si>
+  <si>
+    <t>Lime production dolomitic</t>
+  </si>
+  <si>
+    <t>CARBONATE_CERAMICS</t>
+  </si>
+  <si>
+    <t>CARBONATE_ASH</t>
+  </si>
+  <si>
+    <t>Carbonate ceramics</t>
+  </si>
+  <si>
+    <t>Carbonate soda ash</t>
   </si>
 </sst>
 </file>
@@ -146,15 +268,45 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -163,6 +315,107 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -182,20 +435,18 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -204,22 +455,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -239,26 +475,24 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -267,33 +501,47 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -303,82 +551,96 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -387,6 +649,15 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF99"/>
+      <color rgb="FF00FFFF"/>
+      <color rgb="FFFF99FF"/>
+      <color rgb="FFCCCCFF"/>
+      <color rgb="FFCCFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -662,16 +933,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -682,46 +953,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527558F0-4A8D-4443-AD36-8FAD442485A9}">
   <sheetPr>
-    <tabColor theme="7"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="B2" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{527558F0-4A8D-4443-AD36-8FAD442485A9}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -730,54 +1006,176 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10336FAD-96EF-445B-ABE5-A417976759BF}">
   <sheetPr>
-    <tabColor theme="5" tint="-0.249977111117893"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="39.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="16"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="12"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="12"/>
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="16"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="16"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
+      <c r="B5" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="24"/>
+      <c r="C6" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="24"/>
+      <c r="C7" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="36"/>
+      <c r="C10" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="24"/>
+      <c r="C11" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="34"/>
+      <c r="C12" s="29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="23"/>
+      <c r="C17" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="32" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{10336FAD-96EF-445B-ABE5-A417976759BF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -785,91 +1183,242 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A61706C-08C6-4E4D-9C0F-F30F77D3ECAF}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="9" t="s">
+      <c r="B3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="B4" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="11" t="s">
+      <c r="B5" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="26" t="s">
         <v>26</v>
       </c>
+      <c r="B14" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>43</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{3A61706C-08C6-4E4D-9C0F-F30F77D3ECAF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000360DE9767CDF0449BF75EAB371D3CB7" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="75cb9a07855af6ac97bd432464ca7c04">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784" xmlns:ns3="081a93ea-d517-42a5-a2b7-457060aa7471" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d1676634304aab9936f6a5a5f53c7423" ns2:_="" ns3:_="">
     <xsd:import namespace="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784"/>
@@ -1092,37 +1641,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2734F73-B82F-41CF-9903-48476C4AD16E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D5F53D0-8C3C-4105-858C-106863FDC569}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8336D53-5B17-4ED9-A126-C626AFBB15C6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D6E82EC-3456-4B11-ABE1-84C230E5EEF9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d55314f-45f1-40c9-9fce-63556e193d03"/>
+    <ds:schemaRef ds:uri="48eed89a-7418-4977-ae3a-838f0fac8ec5"/>
+    <ds:schemaRef ds:uri="416d42ac-85ec-40c4-8054-6c816fd4b6a7"/>
+    <ds:schemaRef ds:uri="a1fcbaaf-06d9-47c4-b3a2-beefbc45d784"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E80F6B1A-CBF0-4F55-B3D6-3EB20D7044D8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4BC811B5-F2E0-4DA9-9004-740A8F0CA49E}"/>
 </file>
</xml_diff>